<commit_message>
Excel template: fill in thin borders for new gender rows' empty cells
Cells beyond the last size on rows 19-22 (e.g. cols 22-30 on the
MENS DENIM row which only has 5 sizes) were missing the thin border
because the previous pass only styled cells we wrote a value into. The
chart's bottom line therefore looked like it stayed under 016 instead
of moving down to 020. Now we copy the row-18 styling for every cell
from col 16 through col 30 on each new row, so the chart borders are
continuous across the full width.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/CP_HEADERS_TEMPLATE.xlsx
+++ b/backend/CP_HEADERS_TEMPLATE.xlsx
@@ -9831,31 +9831,38 @@
           <t>5-6</t>
         </is>
       </c>
-      <c r="S19" s="44" t="inlineStr">
+      <c r="S19" s="5" t="inlineStr">
         <is>
           <t>7-8</t>
         </is>
       </c>
-      <c r="T19" s="44" t="inlineStr">
+      <c r="T19" s="5" t="inlineStr">
         <is>
           <t>9-10</t>
         </is>
       </c>
-      <c r="U19" s="44" t="inlineStr">
+      <c r="U19" s="5" t="inlineStr">
         <is>
           <t>11-12</t>
         </is>
       </c>
-      <c r="V19" s="44" t="inlineStr">
+      <c r="V19" s="5" t="inlineStr">
         <is>
           <t>13-14</t>
         </is>
       </c>
-      <c r="W19" s="44" t="inlineStr">
+      <c r="W19" s="5" t="inlineStr">
         <is>
           <t>15-16</t>
         </is>
       </c>
+      <c r="X19" s="5" t="n"/>
+      <c r="Y19" s="5" t="n"/>
+      <c r="Z19" s="5" t="n"/>
+      <c r="AA19" s="5" t="n"/>
+      <c r="AB19" s="5" t="n"/>
+      <c r="AC19" s="5" t="n"/>
+      <c r="AD19" s="5" t="n"/>
     </row>
     <row r="20" ht="16.5" customHeight="1">
       <c r="P20" s="37" t="inlineStr">
@@ -9873,16 +9880,26 @@
           <t>K 3-6</t>
         </is>
       </c>
-      <c r="S20" s="44" t="inlineStr">
+      <c r="S20" s="5" t="inlineStr">
         <is>
           <t>A 3-6</t>
         </is>
       </c>
-      <c r="T20" s="44" t="inlineStr">
+      <c r="T20" s="5" t="inlineStr">
         <is>
           <t>A 7-11</t>
         </is>
       </c>
+      <c r="U20" s="5" t="n"/>
+      <c r="V20" s="5" t="n"/>
+      <c r="W20" s="5" t="n"/>
+      <c r="X20" s="5" t="n"/>
+      <c r="Y20" s="5" t="n"/>
+      <c r="Z20" s="5" t="n"/>
+      <c r="AA20" s="5" t="n"/>
+      <c r="AB20" s="5" t="n"/>
+      <c r="AC20" s="5" t="n"/>
+      <c r="AD20" s="5" t="n"/>
     </row>
     <row r="21" ht="16.5" customHeight="1">
       <c r="P21" s="37" t="inlineStr">
@@ -9900,16 +9917,26 @@
           <t>6-12M</t>
         </is>
       </c>
-      <c r="S21" s="44" t="inlineStr">
+      <c r="S21" s="5" t="inlineStr">
         <is>
           <t>12-18M</t>
         </is>
       </c>
-      <c r="T21" s="44" t="inlineStr">
+      <c r="T21" s="5" t="inlineStr">
         <is>
           <t>18-24M</t>
         </is>
       </c>
+      <c r="U21" s="5" t="n"/>
+      <c r="V21" s="5" t="n"/>
+      <c r="W21" s="5" t="n"/>
+      <c r="X21" s="5" t="n"/>
+      <c r="Y21" s="5" t="n"/>
+      <c r="Z21" s="5" t="n"/>
+      <c r="AA21" s="5" t="n"/>
+      <c r="AB21" s="5" t="n"/>
+      <c r="AC21" s="5" t="n"/>
+      <c r="AD21" s="5" t="n"/>
     </row>
     <row r="22" ht="16.5" customHeight="1">
       <c r="P22" s="37" t="inlineStr">
@@ -9927,21 +9954,30 @@
           <t>30</t>
         </is>
       </c>
-      <c r="S22" s="44" t="inlineStr">
+      <c r="S22" s="5" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="T22" s="44" t="inlineStr">
+      <c r="T22" s="5" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="U22" s="44" t="inlineStr">
+      <c r="U22" s="5" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
+      <c r="V22" s="5" t="n"/>
+      <c r="W22" s="5" t="n"/>
+      <c r="X22" s="5" t="n"/>
+      <c r="Y22" s="5" t="n"/>
+      <c r="Z22" s="5" t="n"/>
+      <c r="AA22" s="5" t="n"/>
+      <c r="AB22" s="5" t="n"/>
+      <c r="AC22" s="5" t="n"/>
+      <c r="AD22" s="5" t="n"/>
     </row>
     <row r="23" ht="16.5" customHeight="1">
       <c r="A23" s="8" t="n">

</xml_diff>